<commit_message>
Republish EU IG with hl7.lt canonical
- Remove EU-specific layout rule from publish-setup.json (wildcard now handles it)
- Rename docs/fhir to docs/eu (correct destination)
- Update feeds with correct canonical URLs (https://hl7.lt/fhir/eu instead of https://hl7.eu/fhir)
- Update all IG content with new canonical and title (HL7 Europe IG Snapshot)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/eu/0.0.1/StructureDefinition-medicalTestResult-eu-core.xlsx
+++ b/docs/eu/0.0.1/StructureDefinition-medicalTestResult-eu-core.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://hl7.eu/fhir/StructureDefinition/medicalTestResult-eu-core</t>
+    <t>https://hl7.lt/fhir/eu/StructureDefinition/medicalTestResult-eu-core</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-15T14:53:25+02:00</t>
+    <t>2026-03-15T17:07:07+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1697,7 +1697,7 @@
     <t>Observation.hasMember</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://hl7.eu/fhir/StructureDefinition/medicalTestResult-eu-core|2.0.0-ballot|QuestionnaireResponse|5.0.0)
+    <t xml:space="preserve">Reference(https://hl7.lt/fhir/eu/StructureDefinition/medicalTestResult-eu-core|2.0.0-ballot|QuestionnaireResponse|5.0.0)
 </t>
   </si>
   <si>
@@ -1719,7 +1719,7 @@
     <t>Observation.derivedFrom</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://hl7.eu/fhir/StructureDefinition/medicalTestResult-eu-core|2.0.0-ballot|ImagingStudy|5.0.0|DocumentReference|5.0.0|QuestionnaireResponse|5.0.0)
+    <t xml:space="preserve">Reference(https://hl7.lt/fhir/eu/StructureDefinition/medicalTestResult-eu-core|2.0.0-ballot|ImagingStudy|5.0.0|DocumentReference|5.0.0|QuestionnaireResponse|5.0.0)
 </t>
   </si>
   <si>

</xml_diff>